<commit_message>
Add audit-log, dashboard, pertinencia and seed data
Introduce audit-log and dashboard modules (controllers, services, DTOs, frontend pages/APIs), a pertinencia validation service (ml/pertinencia_service.py + /validar-pertinencia endpoint), and ML change to return base_value. Add DB DDLs and seed scripts (objeciones_linea_real, reglas_pertinencia_clinica, view vista_tasa_rechazo_codigo, retention migration, base_value column, many seeds). Planillas: add preview, download ZIP of individuales, and Derecho al Olvido flow (logs + MinIO delete). Fix Excel/ExcelJS formatting issues, SHAP/base_value plumbing, predicciones enhancements (tasa rechazos historic), and frontend updates (dashboard, audit UI, CSV export, recharts dependency). Misc: app.module entity/import fixes and enum addition for DERECHO_OLVIDO.
</commit_message>
<xml_diff>
--- a/backend/uploads/consolidadas/EMERGENCIA/Planilla_EMERGENCIA_CONSOLIDADA.xlsx
+++ b/backend/uploads/consolidadas/EMERGENCIA/Planilla_EMERGENCIA_CONSOLIDADA.xlsx
@@ -54,7 +54,7 @@
     <t>Mes y año de prestación:</t>
   </si>
   <si>
-    <t>AGOSTO 2026</t>
+    <t>DICIEMBRE 2026</t>
   </si>
   <si>
     <t>No. Expedientes:</t>
@@ -78,6 +78,12 @@
     <t/>
   </si>
   <si>
+    <t>1701141028</t>
+  </si>
+  <si>
+    <t>CHILIG CHANGOLUISA MARIA ROSA</t>
+  </si>
+  <si>
     <t>1716560089</t>
   </si>
   <si>
@@ -132,12 +138,6 @@
     <t>VALENCIA YUGSI CAMILA ALEJANDRA</t>
   </si>
   <si>
-    <t>1701141028</t>
-  </si>
-  <si>
-    <t>CHILIG CHANGOLUISA MARIA ROSA</t>
-  </si>
-  <si>
     <t>TOTAL VALOR SOLICITADO</t>
   </si>
   <si>
@@ -159,7 +159,7 @@
     <t>CARGO:</t>
   </si>
   <si>
-    <t>ANALISTA - FACTURACIÓN</t>
+    <t>ANALISTA - FACTURACION</t>
   </si>
   <si>
     <t>APROBADO: Econ. Ximena Cobos</t>
@@ -364,7 +364,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -501,9 +501,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1010,7 +1021,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="22">
-        <v>46263.087346886576</v>
+        <v>46279.753973645835</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1030,7 +1041,7 @@
       </c>
       <c r="B9" s="24"/>
       <c r="C9" s="25">
-        <v>206.16</v>
+        <v>269.36</v>
       </c>
       <c r="D9" s="26"/>
       <c r="E9" s="27"/>
@@ -1096,7 +1107,7 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="35">
+      <c r="A16" s="36">
         <v>1</v>
       </c>
       <c r="B16" s="35" t="s">
@@ -1108,12 +1119,12 @@
       <c r="D16" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="35">
-        <v>22.72</v>
+      <c r="E16" s="37">
+        <v>24.87</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="35">
+      <c r="A17" s="36">
         <v>2</v>
       </c>
       <c r="B17" s="35" t="s">
@@ -1125,491 +1136,491 @@
       <c r="D17" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="35">
+      <c r="E17" s="37">
+        <v>22.72</v>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="36">
+        <v>3</v>
+      </c>
+      <c r="B18" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="39">
         <v>20.85</v>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="35">
-        <v>3</v>
-      </c>
-      <c r="B18" s="36" t="s">
+    <row r="19" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="36">
+        <v>4</v>
+      </c>
+      <c r="B19" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="E18" s="36">
+      <c r="C19" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="39">
         <v>20.71</v>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="35">
-        <v>4</v>
-      </c>
-      <c r="B19" s="36" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" s="36" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="36" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="36">
-        <v>29.14</v>
-      </c>
-    </row>
     <row r="20" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="35">
+      <c r="A20" s="36">
         <v>5</v>
       </c>
       <c r="B20" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="36" t="s">
+      <c r="C20" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="36" t="s">
+      <c r="D20" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="36">
-        <v>30.080000000000002</v>
+      <c r="E20" s="39">
+        <v>29.14</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="35">
+      <c r="A21" s="36">
         <v>6</v>
       </c>
       <c r="B21" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="36" t="s">
+      <c r="D21" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="36">
-        <v>29.160000000000004</v>
+      <c r="E21" s="39">
+        <v>30.080000000000002</v>
       </c>
     </row>
     <row r="22" ht="36.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="35">
+      <c r="A22" s="36">
         <v>7</v>
       </c>
       <c r="B22" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="36" t="s">
+      <c r="C22" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="36" t="s">
+      <c r="D22" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="36">
-        <v>14.3</v>
+      <c r="E22" s="39">
+        <v>29.160000000000004</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="35">
+      <c r="A23" s="36">
         <v>8</v>
       </c>
       <c r="B23" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C23" s="36" t="s">
+      <c r="C23" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="36" t="s">
+      <c r="D23" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="36">
-        <v>12.73</v>
+      <c r="E23" s="39">
+        <v>14.3</v>
       </c>
     </row>
     <row r="24" ht="32.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="35">
+      <c r="A24" s="36">
         <v>9</v>
       </c>
       <c r="B24" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C24" s="36" t="s">
+      <c r="C24" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="D24" s="36" t="s">
+      <c r="D24" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="E24" s="36">
-        <v>1.6</v>
+      <c r="E24" s="39">
+        <v>12.73</v>
       </c>
     </row>
     <row r="25" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="35">
+      <c r="A25" s="36">
         <v>10</v>
       </c>
       <c r="B25" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="C25" s="36" t="s">
+      <c r="C25" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="D25" s="36" t="s">
+      <c r="D25" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="36">
-        <v>24.87</v>
+      <c r="E25" s="39">
+        <v>64.8</v>
       </c>
     </row>
     <row r="26" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="35"/>
       <c r="B26" s="35"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="36"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
     </row>
     <row r="27" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="35"/>
       <c r="B27" s="35"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="36"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
     </row>
     <row r="28" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="35"/>
       <c r="B28" s="35"/>
-      <c r="C28" s="37"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="36"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
     </row>
     <row r="29" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="35"/>
       <c r="B29" s="35"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="36"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
     </row>
     <row r="30" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="35"/>
       <c r="B30" s="35"/>
-      <c r="C30" s="37"/>
-      <c r="D30" s="36"/>
-      <c r="E30" s="36"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
     </row>
     <row r="31" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="35"/>
       <c r="B31" s="35"/>
-      <c r="C31" s="37"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="36"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
     </row>
     <row r="32" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="35"/>
       <c r="B32" s="35"/>
-      <c r="C32" s="37"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
     </row>
     <row r="33" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="35"/>
       <c r="B33" s="35"/>
-      <c r="C33" s="37"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="36"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
     </row>
     <row r="34" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="35"/>
       <c r="B34" s="35"/>
-      <c r="C34" s="37"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="36"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
     </row>
     <row r="35" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="35"/>
       <c r="B35" s="35"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="36"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
     </row>
     <row r="36" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="35"/>
       <c r="B36" s="35"/>
-      <c r="C36" s="37"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="36"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
     </row>
     <row r="37" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="35"/>
       <c r="B37" s="35"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="36"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
     </row>
     <row r="38" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="35"/>
       <c r="B38" s="35"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="36"/>
-      <c r="E38" s="36"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
     </row>
     <row r="39" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="35"/>
       <c r="B39" s="35"/>
-      <c r="C39" s="37"/>
-      <c r="D39" s="36"/>
-      <c r="E39" s="36"/>
+      <c r="C39" s="40"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
     </row>
     <row r="40" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="35"/>
       <c r="B40" s="35"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="36"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
     </row>
     <row r="41" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="35"/>
       <c r="B41" s="35"/>
-      <c r="C41" s="37"/>
-      <c r="D41" s="36"/>
-      <c r="E41" s="36"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
     </row>
     <row r="42" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="35"/>
       <c r="B42" s="35"/>
-      <c r="C42" s="37"/>
-      <c r="D42" s="36"/>
-      <c r="E42" s="36"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
     </row>
     <row r="43" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="35"/>
       <c r="B43" s="35"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="36"/>
-      <c r="E43" s="36"/>
+      <c r="C43" s="40"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
     </row>
     <row r="44" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="35"/>
       <c r="B44" s="35"/>
-      <c r="C44" s="37"/>
-      <c r="D44" s="36"/>
-      <c r="E44" s="36"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
     </row>
     <row r="45" ht="21.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="35"/>
       <c r="B45" s="35"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="36"/>
-      <c r="E45" s="36"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="38"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="38"/>
-      <c r="E46" s="39">
-        <v>206.16</v>
+      <c r="B46" s="41"/>
+      <c r="E46" s="42">
+        <v>269.36</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="40"/>
-      <c r="B48" s="40"/>
-      <c r="C48" s="40"/>
-      <c r="D48" s="40"/>
-      <c r="E48" s="40"/>
+      <c r="A48" s="43"/>
+      <c r="B48" s="43"/>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="40"/>
-      <c r="B49" s="40"/>
-      <c r="C49" s="40"/>
-      <c r="D49" s="40"/>
-      <c r="E49" s="40"/>
+      <c r="A49" s="43"/>
+      <c r="B49" s="43"/>
+      <c r="C49" s="43"/>
+      <c r="D49" s="43"/>
+      <c r="E49" s="43"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="40"/>
-      <c r="B50" s="40"/>
-      <c r="C50" s="40"/>
-      <c r="D50" s="40"/>
-      <c r="E50" s="40"/>
+      <c r="A50" s="43"/>
+      <c r="B50" s="43"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="43"/>
+      <c r="E50" s="43"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="40"/>
-      <c r="B51" s="40"/>
-      <c r="C51" s="41"/>
-      <c r="D51" s="41"/>
-      <c r="E51" s="42"/>
+      <c r="A51" s="43"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="44"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="45"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="40"/>
-      <c r="B52" s="40"/>
-      <c r="C52" s="40"/>
-      <c r="D52" s="40"/>
-      <c r="E52" s="40"/>
+      <c r="A52" s="43"/>
+      <c r="B52" s="43"/>
+      <c r="C52" s="43"/>
+      <c r="D52" s="43"/>
+      <c r="E52" s="43"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="40"/>
-      <c r="B53" s="40"/>
-      <c r="C53" s="40"/>
-      <c r="D53" s="40"/>
-      <c r="E53" s="40"/>
+      <c r="A53" s="43"/>
+      <c r="B53" s="43"/>
+      <c r="C53" s="43"/>
+      <c r="D53" s="43"/>
+      <c r="E53" s="43"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="40"/>
-      <c r="B54" s="40"/>
-      <c r="C54" s="40"/>
-      <c r="D54" s="40"/>
-      <c r="E54" s="40"/>
+      <c r="A54" s="43"/>
+      <c r="B54" s="43"/>
+      <c r="C54" s="43"/>
+      <c r="D54" s="43"/>
+      <c r="E54" s="43"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="40"/>
-      <c r="B55" s="40"/>
-      <c r="C55" s="40"/>
-      <c r="D55" s="40"/>
-      <c r="E55" s="40"/>
+      <c r="A55" s="43"/>
+      <c r="B55" s="43"/>
+      <c r="C55" s="43"/>
+      <c r="D55" s="43"/>
+      <c r="E55" s="43"/>
     </row>
     <row r="56" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="43" t="s">
+      <c r="A56" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B56" s="44"/>
-      <c r="C56" s="45" t="s">
+      <c r="B56" s="47"/>
+      <c r="C56" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="D56" s="44"/>
-      <c r="E56" s="44"/>
+      <c r="D56" s="47"/>
+      <c r="E56" s="47"/>
     </row>
     <row r="57" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="46" t="s">
+      <c r="A57" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="B57" s="44"/>
-      <c r="C57" s="47" t="s">
+      <c r="B57" s="47"/>
+      <c r="C57" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="D57" s="48" t="s">
+      <c r="D57" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="E57" s="49"/>
+      <c r="E57" s="52"/>
     </row>
     <row r="58" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="43" t="s">
+      <c r="A58" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="44"/>
-      <c r="C58" s="43" t="s">
+      <c r="B58" s="47"/>
+      <c r="C58" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D58" s="44"/>
-      <c r="E58" s="44"/>
+      <c r="D58" s="47"/>
+      <c r="E58" s="47"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="40"/>
-      <c r="B59" s="40"/>
-      <c r="C59" s="40"/>
-      <c r="D59" s="40"/>
-      <c r="E59" s="40"/>
+      <c r="A59" s="43"/>
+      <c r="B59" s="43"/>
+      <c r="C59" s="43"/>
+      <c r="D59" s="43"/>
+      <c r="E59" s="43"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="40"/>
-      <c r="B60" s="40"/>
-      <c r="C60" s="40"/>
-      <c r="D60" s="40"/>
-      <c r="E60" s="40"/>
+      <c r="A60" s="43"/>
+      <c r="B60" s="43"/>
+      <c r="C60" s="43"/>
+      <c r="D60" s="43"/>
+      <c r="E60" s="43"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="40"/>
-      <c r="B61" s="40"/>
-      <c r="C61" s="40"/>
-      <c r="D61" s="40"/>
-      <c r="E61" s="40"/>
+      <c r="A61" s="43"/>
+      <c r="B61" s="43"/>
+      <c r="C61" s="43"/>
+      <c r="D61" s="43"/>
+      <c r="E61" s="43"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="40"/>
-      <c r="B62" s="40"/>
-      <c r="C62" s="40"/>
-      <c r="D62" s="40"/>
-      <c r="E62" s="40"/>
+      <c r="A62" s="43"/>
+      <c r="B62" s="43"/>
+      <c r="C62" s="43"/>
+      <c r="D62" s="43"/>
+      <c r="E62" s="43"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="40"/>
-      <c r="B63" s="40"/>
-      <c r="C63" s="40"/>
-      <c r="D63" s="40"/>
-      <c r="E63" s="40"/>
+      <c r="A63" s="43"/>
+      <c r="B63" s="43"/>
+      <c r="C63" s="43"/>
+      <c r="D63" s="43"/>
+      <c r="E63" s="43"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="40"/>
-      <c r="B64" s="40"/>
-      <c r="C64" s="40"/>
-      <c r="D64" s="40"/>
-      <c r="E64" s="40"/>
+      <c r="A64" s="43"/>
+      <c r="B64" s="43"/>
+      <c r="C64" s="43"/>
+      <c r="D64" s="43"/>
+      <c r="E64" s="43"/>
     </row>
     <row r="65" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="43" t="s">
+      <c r="A65" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B65" s="44"/>
-      <c r="C65" s="45" t="s">
+      <c r="B65" s="47"/>
+      <c r="C65" s="48" t="s">
         <v>45</v>
       </c>
-      <c r="D65" s="44"/>
-      <c r="E65" s="44"/>
+      <c r="D65" s="47"/>
+      <c r="E65" s="47"/>
     </row>
     <row r="66" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="46" t="s">
+      <c r="A66" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="B66" s="44"/>
-      <c r="C66" s="47" t="s">
+      <c r="B66" s="47"/>
+      <c r="C66" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="D66" s="44"/>
-      <c r="E66" s="44"/>
+      <c r="D66" s="47"/>
+      <c r="E66" s="47"/>
     </row>
     <row r="67" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="43" t="s">
+      <c r="A67" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="B67" s="44"/>
-      <c r="C67" s="43" t="s">
+      <c r="B67" s="47"/>
+      <c r="C67" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="D67" s="48" t="s">
+      <c r="D67" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="E67" s="49"/>
+      <c r="E67" s="52"/>
     </row>
     <row r="68" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="50"/>
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
-      <c r="D68" s="50"/>
-      <c r="E68" s="50"/>
+      <c r="A68" s="53"/>
+      <c r="B68" s="53"/>
+      <c r="C68" s="53"/>
+      <c r="D68" s="53"/>
+      <c r="E68" s="53"/>
     </row>
     <row r="69" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="50"/>
-      <c r="B69" s="50"/>
-      <c r="C69" s="50"/>
-      <c r="D69" s="50"/>
-      <c r="E69" s="50"/>
+      <c r="A69" s="53"/>
+      <c r="B69" s="53"/>
+      <c r="C69" s="53"/>
+      <c r="D69" s="53"/>
+      <c r="E69" s="53"/>
     </row>
     <row r="70" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="50"/>
-      <c r="B70" s="50"/>
-      <c r="C70" s="50"/>
-      <c r="D70" s="50"/>
-      <c r="E70" s="50"/>
+      <c r="A70" s="53"/>
+      <c r="B70" s="53"/>
+      <c r="C70" s="53"/>
+      <c r="D70" s="53"/>
+      <c r="E70" s="53"/>
     </row>
     <row r="71" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="50"/>
-      <c r="B71" s="50"/>
-      <c r="C71" s="50"/>
-      <c r="D71" s="50"/>
-      <c r="E71" s="50"/>
+      <c r="A71" s="53"/>
+      <c r="B71" s="53"/>
+      <c r="C71" s="53"/>
+      <c r="D71" s="53"/>
+      <c r="E71" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>